<commit_message>
Update: Fixed Storage Tanks, Tank Queue and Scheduler
</commit_message>
<xml_diff>
--- a/APPT/data/output/Final Production Plan 2026-01-07.xlsx
+++ b/APPT/data/output/Final Production Plan 2026-01-07.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="528" uniqueCount="239">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="540" uniqueCount="240">
   <si>
     <t>Batch ID</t>
   </si>
@@ -104,15 +104,15 @@
     <t>B016</t>
   </si>
   <si>
+    <t>REP36</t>
+  </si>
+  <si>
     <t>B034</t>
   </si>
   <si>
     <t>B024</t>
   </si>
   <si>
-    <t>REP36</t>
-  </si>
-  <si>
     <t>B017</t>
   </si>
   <si>
@@ -122,33 +122,36 @@
     <t>B018</t>
   </si>
   <si>
+    <t>REP37</t>
+  </si>
+  <si>
     <t>B019</t>
   </si>
   <si>
     <t>B020</t>
   </si>
   <si>
-    <t>REP37</t>
-  </si>
-  <si>
     <t>B021</t>
   </si>
   <si>
     <t>REP38</t>
   </si>
   <si>
+    <t>REP39</t>
+  </si>
+  <si>
     <t>B025</t>
   </si>
   <si>
-    <t>REP39</t>
-  </si>
-  <si>
     <t>REP40</t>
   </si>
   <si>
     <t>B028</t>
   </si>
   <si>
+    <t>REP41</t>
+  </si>
+  <si>
     <t>B030</t>
   </si>
   <si>
@@ -176,15 +179,15 @@
     <t>21417344</t>
   </si>
   <si>
+    <t>95619314</t>
+  </si>
+  <si>
     <t>UNKNOWN</t>
   </si>
   <si>
     <t>'21302239</t>
   </si>
   <si>
-    <t>95619314</t>
-  </si>
-  <si>
     <t>21302239</t>
   </si>
   <si>
@@ -224,15 +227,15 @@
     <t>H&amp;S SHM 72ML X 48 AHF IN GST</t>
   </si>
   <si>
+    <t>Auto-Replenishment HC Base</t>
+  </si>
+  <si>
     <t>PNTN 3MM BIOTIN COND 200MLX24 IN</t>
   </si>
   <si>
     <t>PNTN SHM 75 ML X 48 HS DR IN GST</t>
   </si>
   <si>
-    <t>Auto-Replenishment HC Base</t>
-  </si>
-  <si>
     <t>PNTN SHM 650ML X 12 HFC GST</t>
   </si>
   <si>
@@ -275,52 +278,52 @@
     <t>6T</t>
   </si>
   <si>
+    <t>TK#_56_#</t>
+  </si>
+  <si>
+    <t>TK#_16_#</t>
+  </si>
+  <si>
+    <t>TK#_12_#</t>
+  </si>
+  <si>
+    <t>NO_TANK</t>
+  </si>
+  <si>
+    <t>TK#_9_#</t>
+  </si>
+  <si>
+    <t>TK#_58_#</t>
+  </si>
+  <si>
     <t>TK#_53_#</t>
   </si>
   <si>
+    <t>TK#_23_#</t>
+  </si>
+  <si>
+    <t>TK#_57_#</t>
+  </si>
+  <si>
+    <t>TK#_24_#</t>
+  </si>
+  <si>
     <t>TK#_14_#</t>
   </si>
   <si>
-    <t>TK#_12_#</t>
-  </si>
-  <si>
-    <t>NO_TANK</t>
-  </si>
-  <si>
-    <t>TK#_9_#</t>
-  </si>
-  <si>
-    <t>TK#_23_#</t>
-  </si>
-  <si>
-    <t>TK#_57_#</t>
-  </si>
-  <si>
-    <t>TK#_24_#</t>
-  </si>
-  <si>
-    <t>TK#_58_#</t>
-  </si>
-  <si>
-    <t>TK#_56_#</t>
-  </si>
-  <si>
     <t>TK#_15_#</t>
   </si>
   <si>
-    <t>TK#_16_#</t>
-  </si>
-  <si>
     <t>LOW: DM5500</t>
   </si>
   <si>
     <t>LOW: SLE3S</t>
   </si>
   <si>
+    <t>LOW: SLS</t>
+  </si>
+  <si>
     <t>UNKNOWN_SKU</t>
-  </si>
-  <si>
-    <t>LOW: SLS</t>
   </si>
   <si>
     <t>Time</t>
@@ -1093,7 +1096,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H41"/>
+  <dimension ref="A1:H42"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:8">
@@ -1127,13 +1130,13 @@
         <v>8</v>
       </c>
       <c r="B2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D2" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="E2" s="2">
         <v>46028.79861111111</v>
@@ -1142,10 +1145,10 @@
         <v>46028.86111111111</v>
       </c>
       <c r="G2" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="H2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -1153,13 +1156,13 @@
         <v>9</v>
       </c>
       <c r="B3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C3" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D3" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="E3" s="2">
         <v>46029.11388888889</v>
@@ -1168,10 +1171,10 @@
         <v>46029.17638888889</v>
       </c>
       <c r="G3" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="H3" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -1179,13 +1182,13 @@
         <v>10</v>
       </c>
       <c r="B4" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C4" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D4" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="E4" s="2">
         <v>46029.28333333333</v>
@@ -1194,10 +1197,10 @@
         <v>46029.34583333333</v>
       </c>
       <c r="G4" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="H4" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -1205,13 +1208,13 @@
         <v>11</v>
       </c>
       <c r="B5" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C5" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D5" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="E5" s="2">
         <v>46029.34583333333</v>
@@ -1220,10 +1223,10 @@
         <v>46029.40833333333</v>
       </c>
       <c r="G5" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="H5" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -1231,13 +1234,13 @@
         <v>12</v>
       </c>
       <c r="B6" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C6" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D6" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="E6" s="2">
         <v>46029.48125</v>
@@ -1246,10 +1249,10 @@
         <v>46029.54375</v>
       </c>
       <c r="G6" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="H6" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -1257,13 +1260,13 @@
         <v>13</v>
       </c>
       <c r="B7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C7" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D7" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="E7" s="2">
         <v>46029.58958333333</v>
@@ -1272,10 +1275,10 @@
         <v>46029.65208333333</v>
       </c>
       <c r="G7" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="H7" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -1283,13 +1286,13 @@
         <v>14</v>
       </c>
       <c r="B8" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C8" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D8" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="E8" s="2">
         <v>46029.66458333333</v>
@@ -1298,10 +1301,10 @@
         <v>46029.72708333333</v>
       </c>
       <c r="G8" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="H8" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -1309,13 +1312,13 @@
         <v>15</v>
       </c>
       <c r="B9" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C9" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D9" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="E9" s="2">
         <v>46029.78611111111</v>
@@ -1327,7 +1330,7 @@
         <v>92</v>
       </c>
       <c r="H9" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -1335,13 +1338,13 @@
         <v>16</v>
       </c>
       <c r="B10" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C10" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D10" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="E10" s="2">
         <v>46029.84861111111</v>
@@ -1350,10 +1353,10 @@
         <v>46029.91111111111</v>
       </c>
       <c r="G10" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="H10" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -1361,13 +1364,13 @@
         <v>17</v>
       </c>
       <c r="B11" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C11" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D11" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="E11" s="2">
         <v>46030.03263888889</v>
@@ -1376,10 +1379,10 @@
         <v>46030.09513888889</v>
       </c>
       <c r="G11" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="H11" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="12" spans="1:8">
@@ -1387,13 +1390,13 @@
         <v>18</v>
       </c>
       <c r="B12" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C12" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D12" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="E12" s="2">
         <v>46030.14583333334</v>
@@ -1402,10 +1405,10 @@
         <v>46030.20833333334</v>
       </c>
       <c r="G12" t="s">
-        <v>86</v>
+        <v>93</v>
       </c>
       <c r="H12" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="13" spans="1:8">
@@ -1413,13 +1416,13 @@
         <v>19</v>
       </c>
       <c r="B13" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C13" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D13" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="E13" s="2">
         <v>46030.20833333334</v>
@@ -1428,10 +1431,10 @@
         <v>46030.27083333334</v>
       </c>
       <c r="G13" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="H13" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="14" spans="1:8">
@@ -1439,13 +1442,13 @@
         <v>20</v>
       </c>
       <c r="B14" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C14" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D14" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="E14" s="2">
         <v>46030.27083333334</v>
@@ -1454,10 +1457,10 @@
         <v>46030.33333333334</v>
       </c>
       <c r="G14" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="H14" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="15" spans="1:8">
@@ -1465,13 +1468,13 @@
         <v>21</v>
       </c>
       <c r="B15" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C15" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D15" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="E15" s="2">
         <v>46030.33333333334</v>
@@ -1480,10 +1483,10 @@
         <v>46030.39583333334</v>
       </c>
       <c r="G15" t="s">
-        <v>87</v>
+        <v>94</v>
       </c>
       <c r="H15" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="16" spans="1:8">
@@ -1491,13 +1494,13 @@
         <v>22</v>
       </c>
       <c r="B16" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C16" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D16" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="E16" s="2">
         <v>46030.39583333334</v>
@@ -1506,10 +1509,10 @@
         <v>46030.45833333334</v>
       </c>
       <c r="G16" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="H16" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="17" spans="1:8">
@@ -1517,13 +1520,13 @@
         <v>23</v>
       </c>
       <c r="B17" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C17" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D17" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="E17" s="2">
         <v>46030.45833333334</v>
@@ -1532,10 +1535,10 @@
         <v>46030.52083333334</v>
       </c>
       <c r="G17" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="H17" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="18" spans="1:8">
@@ -1543,13 +1546,13 @@
         <v>24</v>
       </c>
       <c r="B18" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C18" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D18" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="E18" s="2">
         <v>46030.52083333334</v>
@@ -1558,10 +1561,10 @@
         <v>46030.58333333334</v>
       </c>
       <c r="G18" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="H18" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="19" spans="1:8">
@@ -1569,13 +1572,13 @@
         <v>25</v>
       </c>
       <c r="B19" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C19" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D19" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="E19" s="2">
         <v>46030.58333333334</v>
@@ -1584,10 +1587,10 @@
         <v>46030.64583333334</v>
       </c>
       <c r="G19" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="H19" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="20" spans="1:8">
@@ -1595,13 +1598,13 @@
         <v>26</v>
       </c>
       <c r="B20" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C20" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D20" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E20" s="2">
         <v>46028.1875</v>
@@ -1613,7 +1616,7 @@
         <v>92</v>
       </c>
       <c r="H20" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="21" spans="1:8">
@@ -1621,13 +1624,13 @@
         <v>27</v>
       </c>
       <c r="B21" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C21" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D21" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E21" s="2">
         <v>46028.45625</v>
@@ -1636,10 +1639,10 @@
         <v>46028.58125</v>
       </c>
       <c r="G21" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="H21" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="22" spans="1:8">
@@ -1647,13 +1650,13 @@
         <v>28</v>
       </c>
       <c r="B22" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C22" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D22" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E22" s="2">
         <v>46028.71527777778</v>
@@ -1662,10 +1665,10 @@
         <v>46028.77777777778</v>
       </c>
       <c r="G22" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="H22" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="23" spans="1:8">
@@ -1673,25 +1676,25 @@
         <v>29</v>
       </c>
       <c r="B23" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C23" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D23" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E23" s="2">
-        <v>46028.8125</v>
+        <v>46028.79166666666</v>
       </c>
       <c r="F23" s="2">
-        <v>46028.875</v>
+        <v>46028.91666666666</v>
       </c>
       <c r="G23" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="H23" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="24" spans="1:8">
@@ -1699,25 +1702,25 @@
         <v>30</v>
       </c>
       <c r="B24" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C24" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D24" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E24" s="2">
-        <v>46028.91666666666</v>
+        <v>46028.95138888889</v>
       </c>
       <c r="F24" s="2">
-        <v>46028.97916666666</v>
+        <v>46029.01388888889</v>
       </c>
       <c r="G24" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="H24" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
     </row>
     <row r="25" spans="1:8">
@@ -1725,25 +1728,25 @@
         <v>31</v>
       </c>
       <c r="B25" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C25" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D25" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E25" s="2">
-        <v>46028.99305555555</v>
+        <v>46029.05555555555</v>
       </c>
       <c r="F25" s="2">
         <v>46029.11805555555</v>
       </c>
       <c r="G25" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="H25" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="26" spans="1:8">
@@ -1751,13 +1754,13 @@
         <v>32</v>
       </c>
       <c r="B26" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C26" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D26" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E26" s="2">
         <v>46029.13194444445</v>
@@ -1766,10 +1769,10 @@
         <v>46029.19097222222</v>
       </c>
       <c r="G26" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="H26" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="27" spans="1:8">
@@ -1777,13 +1780,13 @@
         <v>33</v>
       </c>
       <c r="B27" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C27" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D27" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E27" s="2">
         <v>46029.22569444445</v>
@@ -1792,10 +1795,10 @@
         <v>46029.28819444445</v>
       </c>
       <c r="G27" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="H27" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
     </row>
     <row r="28" spans="1:8">
@@ -1803,13 +1806,13 @@
         <v>34</v>
       </c>
       <c r="B28" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C28" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D28" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E28" s="2">
         <v>46029.32986111111</v>
@@ -1818,10 +1821,10 @@
         <v>46029.39236111111</v>
       </c>
       <c r="G28" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="H28" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="29" spans="1:8">
@@ -1829,25 +1832,25 @@
         <v>35</v>
       </c>
       <c r="B29" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="C29" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="D29" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E29" s="2">
         <v>46029.40625</v>
       </c>
       <c r="F29" s="2">
-        <v>46029.46875</v>
+        <v>46029.53125</v>
       </c>
       <c r="G29" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="H29" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
     <row r="30" spans="1:8">
@@ -1855,25 +1858,25 @@
         <v>36</v>
       </c>
       <c r="B30" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C30" t="s">
         <v>76</v>
       </c>
       <c r="D30" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E30" s="2">
-        <v>46029.46875</v>
+        <v>46029.54513888889</v>
       </c>
       <c r="F30" s="2">
-        <v>46029.53125</v>
+        <v>46029.60763888889</v>
       </c>
       <c r="G30" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="H30" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="31" spans="1:8">
@@ -1881,25 +1884,25 @@
         <v>37</v>
       </c>
       <c r="B31" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="C31" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="D31" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E31" s="2">
-        <v>46029.54513888889</v>
+        <v>46029.60763888889</v>
       </c>
       <c r="F31" s="2">
         <v>46029.67013888889</v>
       </c>
       <c r="G31" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="H31" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="32" spans="1:8">
@@ -1907,13 +1910,13 @@
         <v>38</v>
       </c>
       <c r="B32" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C32" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D32" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E32" s="2">
         <v>46029.68402777778</v>
@@ -1922,10 +1925,10 @@
         <v>46029.74305555555</v>
       </c>
       <c r="G32" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="H32" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="33" spans="1:8">
@@ -1933,22 +1936,22 @@
         <v>39</v>
       </c>
       <c r="B33" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C33" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D33" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E33" s="2">
-        <v>46029.92638888889</v>
+        <v>46029.84097222222</v>
       </c>
       <c r="F33" s="2">
-        <v>46030.05138888889</v>
+        <v>46029.96597222222</v>
       </c>
       <c r="G33" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="H33" t="s">
         <v>101</v>
@@ -1959,25 +1962,25 @@
         <v>40</v>
       </c>
       <c r="B34" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="C34" t="s">
-        <v>78</v>
+        <v>70</v>
       </c>
       <c r="D34" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E34" s="2">
-        <v>46030.06527777778</v>
+        <v>46029.96597222222</v>
       </c>
       <c r="F34" s="2">
-        <v>46030.12777777778</v>
+        <v>46030.09097222222</v>
       </c>
       <c r="G34" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="H34" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
     <row r="35" spans="1:8">
@@ -1985,25 +1988,25 @@
         <v>41</v>
       </c>
       <c r="B35" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="C35" t="s">
-        <v>71</v>
+        <v>79</v>
       </c>
       <c r="D35" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E35" s="2">
-        <v>46030.14166666667</v>
+        <v>46030.10486111111</v>
       </c>
       <c r="F35" s="2">
-        <v>46030.26666666667</v>
+        <v>46030.16736111111</v>
       </c>
       <c r="G35" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="H35" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="36" spans="1:8">
@@ -2011,22 +2014,22 @@
         <v>42</v>
       </c>
       <c r="B36" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C36" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D36" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E36" s="2">
-        <v>46030.26666666667</v>
+        <v>46030.23194444444</v>
       </c>
       <c r="F36" s="2">
-        <v>46030.39166666667</v>
+        <v>46030.35694444444</v>
       </c>
       <c r="G36" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="H36" t="s">
         <v>101</v>
@@ -2037,25 +2040,25 @@
         <v>43</v>
       </c>
       <c r="B37" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C37" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D37" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E37" s="2">
-        <v>46030.40555555555</v>
+        <v>46030.37083333333</v>
       </c>
       <c r="F37" s="2">
-        <v>46030.46805555555</v>
+        <v>46030.43333333333</v>
       </c>
       <c r="G37" t="s">
-        <v>86</v>
+        <v>95</v>
       </c>
       <c r="H37" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="38" spans="1:8">
@@ -2063,25 +2066,25 @@
         <v>44</v>
       </c>
       <c r="B38" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="C38" t="s">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="D38" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E38" s="2">
-        <v>46030.58611111111</v>
+        <v>46030.44722222222</v>
       </c>
       <c r="F38" s="2">
-        <v>46030.64861111111</v>
+        <v>46030.57222222222</v>
       </c>
       <c r="G38" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="H38" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
     <row r="39" spans="1:8">
@@ -2089,25 +2092,25 @@
         <v>45</v>
       </c>
       <c r="B39" t="s">
-        <v>60</v>
+        <v>51</v>
       </c>
       <c r="C39" t="s">
         <v>81</v>
       </c>
       <c r="D39" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E39" s="2">
-        <v>46030.67708333334</v>
+        <v>46030.58611111111</v>
       </c>
       <c r="F39" s="2">
-        <v>46030.73611111111</v>
+        <v>46030.64861111111</v>
       </c>
       <c r="G39" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="H39" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="40" spans="1:8">
@@ -2121,19 +2124,19 @@
         <v>82</v>
       </c>
       <c r="D40" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E40" s="2">
-        <v>46030.75</v>
+        <v>46030.67708333334</v>
       </c>
       <c r="F40" s="2">
-        <v>46030.80902777778</v>
+        <v>46030.73611111111</v>
       </c>
       <c r="G40" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="H40" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="41" spans="1:8">
@@ -2141,25 +2144,51 @@
         <v>47</v>
       </c>
       <c r="B41" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="C41" t="s">
         <v>83</v>
       </c>
       <c r="D41" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E41" s="2">
+        <v>46030.75</v>
+      </c>
+      <c r="F41" s="2">
+        <v>46030.80902777778</v>
+      </c>
+      <c r="G41" t="s">
+        <v>87</v>
+      </c>
+      <c r="H41" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8">
+      <c r="A42" t="s">
+        <v>48</v>
+      </c>
+      <c r="B42" t="s">
+        <v>57</v>
+      </c>
+      <c r="C42" t="s">
+        <v>84</v>
+      </c>
+      <c r="D42" t="s">
+        <v>86</v>
+      </c>
+      <c r="E42" s="2">
         <v>46030.82291666666</v>
       </c>
-      <c r="F41" s="2">
+      <c r="F42" s="2">
         <v>46030.88194444445</v>
       </c>
-      <c r="G41" t="s">
-        <v>96</v>
-      </c>
-      <c r="H41" t="s">
-        <v>98</v>
+      <c r="G42" t="s">
+        <v>97</v>
+      </c>
+      <c r="H42" t="s">
+        <v>99</v>
       </c>
     </row>
   </sheetData>
@@ -2174,26 +2203,26 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C3" t="s">
         <v>26</v>
@@ -2201,7 +2230,7 @@
     </row>
     <row r="4" spans="1:4">
       <c r="A4" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C4" t="s">
         <v>26</v>
@@ -2209,7 +2238,7 @@
     </row>
     <row r="5" spans="1:4">
       <c r="A5" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C5" t="s">
         <v>26</v>
@@ -2217,7 +2246,7 @@
     </row>
     <row r="6" spans="1:4">
       <c r="A6" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C6" t="s">
         <v>26</v>
@@ -2225,7 +2254,7 @@
     </row>
     <row r="7" spans="1:4">
       <c r="A7" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C7" t="s">
         <v>26</v>
@@ -2233,7 +2262,7 @@
     </row>
     <row r="8" spans="1:4">
       <c r="A8" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C8" t="s">
         <v>26</v>
@@ -2241,42 +2270,42 @@
     </row>
     <row r="9" spans="1:4">
       <c r="A9" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="11" spans="1:4">
       <c r="A11" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="12" spans="1:4">
       <c r="A12" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="13" spans="1:4">
       <c r="A13" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="14" spans="1:4">
       <c r="A14" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="15" spans="1:4">
       <c r="A15" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="16" spans="1:4">
       <c r="A16" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C16" t="s">
         <v>27</v>
@@ -2284,7 +2313,7 @@
     </row>
     <row r="17" spans="1:3">
       <c r="A17" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C17" t="s">
         <v>27</v>
@@ -2292,7 +2321,7 @@
     </row>
     <row r="18" spans="1:3">
       <c r="A18" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C18" t="s">
         <v>27</v>
@@ -2300,7 +2329,7 @@
     </row>
     <row r="19" spans="1:3">
       <c r="A19" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C19" t="s">
         <v>27</v>
@@ -2308,7 +2337,7 @@
     </row>
     <row r="20" spans="1:3">
       <c r="A20" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C20" t="s">
         <v>27</v>
@@ -2316,7 +2345,7 @@
     </row>
     <row r="21" spans="1:3">
       <c r="A21" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C21" t="s">
         <v>27</v>
@@ -2324,42 +2353,42 @@
     </row>
     <row r="22" spans="1:3">
       <c r="A22" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
     </row>
     <row r="23" spans="1:3">
       <c r="A23" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="24" spans="1:3">
       <c r="A24" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
     </row>
     <row r="25" spans="1:3">
       <c r="A25" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
     </row>
     <row r="26" spans="1:3">
       <c r="A26" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
     </row>
     <row r="27" spans="1:3">
       <c r="A27" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="28" spans="1:3">
       <c r="A28" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
     </row>
     <row r="29" spans="1:3">
       <c r="A29" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C29" t="s">
         <v>28</v>
@@ -2367,7 +2396,7 @@
     </row>
     <row r="30" spans="1:3">
       <c r="A30" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C30" t="s">
         <v>28</v>
@@ -2375,7 +2404,7 @@
     </row>
     <row r="31" spans="1:3">
       <c r="A31" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C31" t="s">
         <v>28</v>
@@ -2383,12 +2412,15 @@
     </row>
     <row r="32" spans="1:3">
       <c r="A32" t="s">
-        <v>134</v>
+        <v>135</v>
+      </c>
+      <c r="C32" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="33" spans="1:3">
       <c r="A33" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B33" t="s">
         <v>8</v>
@@ -2399,7 +2431,7 @@
     </row>
     <row r="34" spans="1:3">
       <c r="A34" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B34" t="s">
         <v>8</v>
@@ -2410,7 +2442,7 @@
     </row>
     <row r="35" spans="1:3">
       <c r="A35" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B35" t="s">
         <v>8</v>
@@ -2421,33 +2453,33 @@
     </row>
     <row r="36" spans="1:3">
       <c r="A36" t="s">
-        <v>138</v>
+        <v>139</v>
+      </c>
+      <c r="C36" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="37" spans="1:3">
       <c r="A37" t="s">
-        <v>139</v>
+        <v>140</v>
+      </c>
+      <c r="C37" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="38" spans="1:3">
       <c r="A38" t="s">
-        <v>140</v>
-      </c>
-      <c r="C38" t="s">
-        <v>30</v>
+        <v>141</v>
       </c>
     </row>
     <row r="39" spans="1:3">
       <c r="A39" t="s">
-        <v>141</v>
-      </c>
-      <c r="C39" t="s">
-        <v>30</v>
+        <v>142</v>
       </c>
     </row>
     <row r="40" spans="1:3">
       <c r="A40" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C40" t="s">
         <v>30</v>
@@ -2455,36 +2487,33 @@
     </row>
     <row r="41" spans="1:3">
       <c r="A41" t="s">
-        <v>143</v>
+        <v>144</v>
+      </c>
+      <c r="C41" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="42" spans="1:3">
       <c r="A42" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C42" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="43" spans="1:3">
       <c r="A43" t="s">
-        <v>145</v>
-      </c>
-      <c r="C43" t="s">
-        <v>31</v>
+        <v>146</v>
       </c>
     </row>
     <row r="44" spans="1:3">
       <c r="A44" t="s">
-        <v>146</v>
-      </c>
-      <c r="C44" t="s">
-        <v>31</v>
+        <v>147</v>
       </c>
     </row>
     <row r="45" spans="1:3">
       <c r="A45" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C45" t="s">
         <v>31</v>
@@ -2492,7 +2521,7 @@
     </row>
     <row r="46" spans="1:3">
       <c r="A46" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C46" t="s">
         <v>31</v>
@@ -2500,7 +2529,7 @@
     </row>
     <row r="47" spans="1:3">
       <c r="A47" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C47" t="s">
         <v>31</v>
@@ -2508,7 +2537,7 @@
     </row>
     <row r="48" spans="1:3">
       <c r="A48" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B48" t="s">
         <v>9</v>
@@ -2516,7 +2545,7 @@
     </row>
     <row r="49" spans="1:3">
       <c r="A49" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B49" t="s">
         <v>9</v>
@@ -2527,7 +2556,7 @@
     </row>
     <row r="50" spans="1:3">
       <c r="A50" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B50" t="s">
         <v>9</v>
@@ -2538,7 +2567,7 @@
     </row>
     <row r="51" spans="1:3">
       <c r="A51" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C51" t="s">
         <v>32</v>
@@ -2546,12 +2575,12 @@
     </row>
     <row r="52" spans="1:3">
       <c r="A52" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
     </row>
     <row r="53" spans="1:3">
       <c r="A53" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="C53" t="s">
         <v>33</v>
@@ -2559,7 +2588,7 @@
     </row>
     <row r="54" spans="1:3">
       <c r="A54" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="C54" t="s">
         <v>33</v>
@@ -2567,7 +2596,7 @@
     </row>
     <row r="55" spans="1:3">
       <c r="A55" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="C55" t="s">
         <v>33</v>
@@ -2575,7 +2604,7 @@
     </row>
     <row r="56" spans="1:3">
       <c r="A56" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="B56" t="s">
         <v>10</v>
@@ -2583,7 +2612,7 @@
     </row>
     <row r="57" spans="1:3">
       <c r="A57" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B57" t="s">
         <v>10</v>
@@ -2591,7 +2620,7 @@
     </row>
     <row r="58" spans="1:3">
       <c r="A58" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B58" t="s">
         <v>10</v>
@@ -2602,7 +2631,7 @@
     </row>
     <row r="59" spans="1:3">
       <c r="A59" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B59" t="s">
         <v>11</v>
@@ -2613,7 +2642,7 @@
     </row>
     <row r="60" spans="1:3">
       <c r="A60" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B60" t="s">
         <v>11</v>
@@ -2624,7 +2653,7 @@
     </row>
     <row r="61" spans="1:3">
       <c r="A61" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="B61" t="s">
         <v>11</v>
@@ -2632,7 +2661,7 @@
     </row>
     <row r="62" spans="1:3">
       <c r="A62" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C62" t="s">
         <v>35</v>
@@ -2640,7 +2669,7 @@
     </row>
     <row r="63" spans="1:3">
       <c r="A63" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="C63" t="s">
         <v>35</v>
@@ -2648,7 +2677,7 @@
     </row>
     <row r="64" spans="1:3">
       <c r="A64" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C64" t="s">
         <v>35</v>
@@ -2656,37 +2685,37 @@
     </row>
     <row r="65" spans="1:3">
       <c r="A65" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="C65" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="66" spans="1:3">
       <c r="A66" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B66" t="s">
         <v>12</v>
       </c>
       <c r="C66" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="67" spans="1:3">
       <c r="A67" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="B67" t="s">
         <v>12</v>
       </c>
       <c r="C67" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="68" spans="1:3">
       <c r="A68" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B68" t="s">
         <v>12</v>
@@ -2694,34 +2723,34 @@
     </row>
     <row r="69" spans="1:3">
       <c r="A69" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C69" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="70" spans="1:3">
       <c r="A70" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C70" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="71" spans="1:3">
       <c r="A71" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="B71" t="s">
         <v>13</v>
       </c>
       <c r="C71" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="72" spans="1:3">
       <c r="A72" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="B72" t="s">
         <v>13</v>
@@ -2732,7 +2761,7 @@
     </row>
     <row r="73" spans="1:3">
       <c r="A73" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B73" t="s">
         <v>13</v>
@@ -2743,7 +2772,7 @@
     </row>
     <row r="74" spans="1:3">
       <c r="A74" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B74" t="s">
         <v>14</v>
@@ -2754,7 +2783,7 @@
     </row>
     <row r="75" spans="1:3">
       <c r="A75" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="B75" t="s">
         <v>14</v>
@@ -2765,7 +2794,7 @@
     </row>
     <row r="76" spans="1:3">
       <c r="A76" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B76" t="s">
         <v>14</v>
@@ -2776,7 +2805,7 @@
     </row>
     <row r="77" spans="1:3">
       <c r="A77" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="C77" t="s">
         <v>38</v>
@@ -2784,17 +2813,17 @@
     </row>
     <row r="78" spans="1:3">
       <c r="A78" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
     </row>
     <row r="79" spans="1:3">
       <c r="A79" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="80" spans="1:3">
       <c r="A80" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B80" t="s">
         <v>15</v>
@@ -2802,7 +2831,7 @@
     </row>
     <row r="81" spans="1:3">
       <c r="A81" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="B81" t="s">
         <v>15</v>
@@ -2810,7 +2839,7 @@
     </row>
     <row r="82" spans="1:3">
       <c r="A82" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B82" t="s">
         <v>15</v>
@@ -2818,36 +2847,48 @@
     </row>
     <row r="83" spans="1:3">
       <c r="A83" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="B83" t="s">
         <v>16</v>
       </c>
+      <c r="C83" t="s">
+        <v>39</v>
+      </c>
     </row>
     <row r="84" spans="1:3">
       <c r="A84" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="B84" t="s">
         <v>16</v>
       </c>
+      <c r="C84" t="s">
+        <v>39</v>
+      </c>
     </row>
     <row r="85" spans="1:3">
       <c r="A85" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="B85" t="s">
         <v>16</v>
       </c>
+      <c r="C85" t="s">
+        <v>39</v>
+      </c>
     </row>
     <row r="86" spans="1:3">
       <c r="A86" t="s">
-        <v>188</v>
+        <v>189</v>
+      </c>
+      <c r="C86" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="87" spans="1:3">
       <c r="A87" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="C87" t="s">
         <v>39</v>
@@ -2855,7 +2896,7 @@
     </row>
     <row r="88" spans="1:3">
       <c r="A88" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="C88" t="s">
         <v>39</v>
@@ -2863,50 +2904,53 @@
     </row>
     <row r="89" spans="1:3">
       <c r="A89" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="C89" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="90" spans="1:3">
       <c r="A90" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="C90" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="91" spans="1:3">
       <c r="A91" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="C91" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="92" spans="1:3">
       <c r="A92" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B92" t="s">
         <v>17</v>
       </c>
       <c r="C92" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="93" spans="1:3">
       <c r="A93" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="B93" t="s">
         <v>17</v>
       </c>
+      <c r="C93" t="s">
+        <v>40</v>
+      </c>
     </row>
     <row r="94" spans="1:3">
       <c r="A94" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B94" t="s">
         <v>17</v>
@@ -2917,23 +2961,20 @@
     </row>
     <row r="95" spans="1:3">
       <c r="A95" t="s">
-        <v>197</v>
-      </c>
-      <c r="C95" t="s">
-        <v>40</v>
+        <v>198</v>
       </c>
     </row>
     <row r="96" spans="1:3">
       <c r="A96" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="C96" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="97" spans="1:3">
       <c r="A97" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="B97" t="s">
         <v>18</v>
@@ -2944,7 +2985,7 @@
     </row>
     <row r="98" spans="1:3">
       <c r="A98" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="B98" t="s">
         <v>18</v>
@@ -2955,51 +2996,42 @@
     </row>
     <row r="99" spans="1:3">
       <c r="A99" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B99" t="s">
         <v>18</v>
       </c>
-      <c r="C99" t="s">
-        <v>41</v>
-      </c>
     </row>
     <row r="100" spans="1:3">
       <c r="A100" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="B100" t="s">
         <v>19</v>
       </c>
-      <c r="C100" t="s">
-        <v>41</v>
-      </c>
     </row>
     <row r="101" spans="1:3">
       <c r="A101" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="B101" t="s">
         <v>19</v>
       </c>
-      <c r="C101" t="s">
-        <v>41</v>
-      </c>
     </row>
     <row r="102" spans="1:3">
       <c r="A102" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="B102" t="s">
         <v>19</v>
       </c>
       <c r="C102" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="103" spans="1:3">
       <c r="A103" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B103" t="s">
         <v>20</v>
@@ -3010,7 +3042,7 @@
     </row>
     <row r="104" spans="1:3">
       <c r="A104" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="B104" t="s">
         <v>20</v>
@@ -3021,7 +3053,7 @@
     </row>
     <row r="105" spans="1:3">
       <c r="A105" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="B105" t="s">
         <v>20</v>
@@ -3032,7 +3064,7 @@
     </row>
     <row r="106" spans="1:3">
       <c r="A106" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="B106" t="s">
         <v>21</v>
@@ -3043,7 +3075,7 @@
     </row>
     <row r="107" spans="1:3">
       <c r="A107" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="B107" t="s">
         <v>21</v>
@@ -3054,26 +3086,29 @@
     </row>
     <row r="108" spans="1:3">
       <c r="A108" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="B108" t="s">
         <v>21</v>
       </c>
       <c r="C108" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="109" spans="1:3">
       <c r="A109" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="B109" t="s">
         <v>22</v>
       </c>
+      <c r="C109" t="s">
+        <v>43</v>
+      </c>
     </row>
     <row r="110" spans="1:3">
       <c r="A110" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="B110" t="s">
         <v>22</v>
@@ -3084,69 +3119,81 @@
     </row>
     <row r="111" spans="1:3">
       <c r="A111" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B111" t="s">
         <v>22</v>
       </c>
-      <c r="C111" t="s">
-        <v>43</v>
-      </c>
     </row>
     <row r="112" spans="1:3">
       <c r="A112" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="B112" t="s">
         <v>23</v>
       </c>
       <c r="C112" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="113" spans="1:3">
       <c r="A113" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B113" t="s">
         <v>23</v>
       </c>
+      <c r="C113" t="s">
+        <v>44</v>
+      </c>
     </row>
     <row r="114" spans="1:3">
       <c r="A114" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="B114" t="s">
         <v>23</v>
       </c>
+      <c r="C114" t="s">
+        <v>44</v>
+      </c>
     </row>
     <row r="115" spans="1:3">
       <c r="A115" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="B115" t="s">
         <v>24</v>
       </c>
+      <c r="C115" t="s">
+        <v>44</v>
+      </c>
     </row>
     <row r="116" spans="1:3">
       <c r="A116" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="B116" t="s">
         <v>24</v>
       </c>
+      <c r="C116" t="s">
+        <v>44</v>
+      </c>
     </row>
     <row r="117" spans="1:3">
       <c r="A117" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="B117" t="s">
         <v>24</v>
       </c>
+      <c r="C117" t="s">
+        <v>44</v>
+      </c>
     </row>
     <row r="118" spans="1:3">
       <c r="A118" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="B118" t="s">
         <v>25</v>
@@ -3154,134 +3201,134 @@
     </row>
     <row r="119" spans="1:3">
       <c r="A119" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="B119" t="s">
         <v>25</v>
       </c>
       <c r="C119" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="120" spans="1:3">
       <c r="A120" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B120" t="s">
         <v>25</v>
       </c>
       <c r="C120" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="121" spans="1:3">
       <c r="A121" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="C121" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="122" spans="1:3">
       <c r="A122" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
     </row>
     <row r="123" spans="1:3">
       <c r="A123" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="C123" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="124" spans="1:3">
       <c r="A124" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="C124" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="125" spans="1:3">
       <c r="A125" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="C125" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="126" spans="1:3">
       <c r="A126" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="C126" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="127" spans="1:3">
       <c r="A127" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="C127" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="128" spans="1:3">
       <c r="A128" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="C128" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="129" spans="1:3">
       <c r="A129" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
     </row>
     <row r="130" spans="1:3">
       <c r="A130" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="C130" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="131" spans="1:3">
       <c r="A131" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="C131" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="132" spans="1:3">
       <c r="A132" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="C132" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="133" spans="1:3">
       <c r="A133" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="134" spans="1:3">
       <c r="A134" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="135" spans="1:3">
       <c r="A135" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
     </row>
     <row r="136" spans="1:3">
       <c r="A136" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
     </row>
   </sheetData>

</xml_diff>